<commit_message>
chore(registers): regenerate all REG-XX with branded BFF-style header
</commit_message>
<xml_diff>
--- a/public/ims/REG-04-Employee-Register.xlsx
+++ b/public/ims/REG-04-Employee-Register.xlsx
@@ -13,12 +13,63 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="94">
-  <si>
-    <t>REG-04 — Employee Register: Active Employees</t>
-  </si>
-  <si>
-    <t>ISO 9001:2015 §7.1.2 | All current human and agentic workers</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="113">
+  <si>
+    <t>TITLE</t>
+  </si>
+  <si>
+    <t>PREQAL EMPLOYEE REGISTER — ACTIVE EMPLOYEES</t>
+  </si>
+  <si>
+    <t>HUMAN</t>
+  </si>
+  <si>
+    <t>CREATED</t>
+  </si>
+  <si>
+    <t>REVISED</t>
+  </si>
+  <si>
+    <t>APPROVED</t>
+  </si>
+  <si>
+    <t>DCN</t>
+  </si>
+  <si>
+    <t>PQL-REG-04</t>
+  </si>
+  <si>
+    <t>AGENTIC</t>
+  </si>
+  <si>
+    <t>SCOPE</t>
+  </si>
+  <si>
+    <t>HUMAN RESOURCES | ISO 9001:2015 §7.1.2</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>CREATION DATE</t>
+  </si>
+  <si>
+    <t>2026-05-14</t>
+  </si>
+  <si>
+    <t>APPROVAL DATE</t>
+  </si>
+  <si>
+    <t>VERSION NUMBER</t>
+  </si>
+  <si>
+    <t>1.0</t>
+  </si>
+  <si>
+    <t>CURRENT REVISION DATE</t>
+  </si>
+  <si>
+    <t>SCHEDULED REVISION DATE</t>
   </si>
   <si>
     <t>Emp ID</t>
@@ -156,10 +207,13 @@
     <t>Claude AI (Anthropic) — SOP-09 authorised</t>
   </si>
   <si>
-    <t>REG-04 — Employee Register: Training Log</t>
-  </si>
-  <si>
-    <t>ISO 9001:2015 §7.2 | Competence and training records</t>
+    <t>PREQAL EMPLOYEE REGISTER — TRAINING LOG</t>
+  </si>
+  <si>
+    <t>TRAINING</t>
+  </si>
+  <si>
+    <t>HUMAN RESOURCES | ISO 9001:2015 §7.2</t>
   </si>
   <si>
     <t>Log ID</t>
@@ -216,10 +270,13 @@
     <t>[Provider]</t>
   </si>
   <si>
-    <t>REG-04 — Employee Register: Role Descriptions</t>
-  </si>
-  <si>
-    <t>ISO 9001:2015 §7.1.2, §7.2 | Defined responsibilities per role</t>
+    <t>PREQAL EMPLOYEE REGISTER — ROLE DESCRIPTIONS</t>
+  </si>
+  <si>
+    <t>ROLES</t>
+  </si>
+  <si>
+    <t>HUMAN RESOURCES | ISO 9001:2015 §7.1.2, §7.2</t>
   </si>
   <si>
     <t>Role ID</t>
@@ -301,7 +358,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+  </numFmts>
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -310,13 +370,35 @@
       <name val="Calibri"/>
     </font>
     <font>
-      <b/>
-      <color rgb="FF0F172A"/>
-      <sz val="14"/>
+      <sz val="10"/>
       <name val="Arial"/>
     </font>
     <font>
-      <color rgb="FF334155"/>
+      <b/>
+      <color rgb="FF0F172A"/>
+      <sz val="36"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="9"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF0F172A"/>
+      <sz val="18"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF0F172A"/>
       <sz val="10"/>
       <name val="Arial"/>
     </font>
@@ -326,8 +408,13 @@
       <sz val="11"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <color rgb="FF334155"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -336,17 +423,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FF0F172A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFEF3C7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
+        <fgColor rgb="FFFFFBEB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF0F172A"/>
+        <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -382,21 +474,38 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -414,6 +523,138 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor editAs="absolute">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>16000</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>71999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="857250" cy="952500"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor editAs="absolute">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>16000</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>71999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="857250" cy="952500"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor editAs="absolute">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>16000</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>71999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="857250" cy="952500"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -738,7 +979,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I11"/>
+  <dimension ref="A2:J19"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -750,279 +991,429 @@
     <col min="7" max="7" width="14" customWidth="1"/>
     <col min="8" max="8" width="12" customWidth="1"/>
     <col min="9" max="9" width="35" customWidth="1"/>
+    <col min="10" max="10" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="2" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-    </row>
-    <row r="2" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-    </row>
-    <row r="4" ht="28" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="E2" s="4">
+        <v>7</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="G2" s="5">
+        <v>1</v>
+      </c>
+      <c r="H2" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="I2" s="6" t="s">
         <v>4</v>
       </c>
+      <c r="J2" s="6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="4"/>
+      <c r="F3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G3" s="5">
+        <v>6</v>
+      </c>
+      <c r="H3" s="7">
+        <v>7</v>
+      </c>
+      <c r="I3" s="7">
+        <v>0</v>
+      </c>
+      <c r="J3" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="2" t="s">
+        <v>9</v>
+      </c>
       <c r="D4" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="I4" s="3" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="5" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="4" t="s">
+      <c r="E4" s="4"/>
+      <c r="F4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H4" s="7"/>
+      <c r="I4" s="7"/>
+      <c r="J4" s="7"/>
+    </row>
+    <row r="5" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="D5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="E5" s="4"/>
+      <c r="F5" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H5" s="7"/>
+      <c r="I5" s="7"/>
+      <c r="J5" s="7"/>
+    </row>
+    <row r="6" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="D6" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" s="4"/>
+      <c r="H6" s="8">
+        <v>1</v>
+      </c>
+      <c r="I6" s="8">
+        <v>0</v>
+      </c>
+      <c r="J6" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="1"/>
+      <c r="B7" s="1"/>
+      <c r="C7" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="D7" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="E7" s="4"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="8"/>
+      <c r="J7" s="8"/>
+    </row>
+    <row r="8" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="1"/>
+      <c r="B8" s="1"/>
+      <c r="C8" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="D8" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" s="4"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+    </row>
+    <row r="9" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="1"/>
+      <c r="B9" s="1"/>
+      <c r="C9" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="I5" s="4" t="s">
+      <c r="D9" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" s="4"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
+    </row>
+    <row r="10" ht="6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="1"/>
+      <c r="B10" s="1"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="9"/>
+      <c r="H10" s="9"/>
+      <c r="I10" s="9"/>
+    </row>
+    <row r="11" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="12" ht="28" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="10" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="6" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
+      <c r="B12" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="C12" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="D12" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="E12" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="F12" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="F6" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="G6" s="5" t="s">
+      <c r="G12" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="H6" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="I6" s="5" t="s">
+      <c r="H12" s="10" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="7" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
+      <c r="I12" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="B7" s="4" t="s">
+    </row>
+    <row r="13" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="C7" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D7" s="4" t="s">
+      <c r="B13" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="E7" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="I7" s="4" t="s">
+      <c r="C13" s="11" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="8" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
+      <c r="D13" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="E13" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="C8" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D8" s="5" t="s">
+      <c r="F13" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="E8" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="H8" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="I8" s="5" t="s">
+      <c r="G13" s="11" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="9" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
+      <c r="H13" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="I13" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="C9" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D9" s="4" t="s">
+    </row>
+    <row r="14" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="E9" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="I9" s="4" t="s">
+      <c r="B14" s="12" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="10" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="5" t="s">
+      <c r="C14" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="D14" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="C10" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D10" s="5" t="s">
+      <c r="E14" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="E10" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="H10" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="I10" s="5" t="s">
+      <c r="F14" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="G14" s="12" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="11" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
+      <c r="H14" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="I14" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="B11" s="4" t="s">
+    </row>
+    <row r="15" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="C11" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D11" s="4" t="s">
+      <c r="B15" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="E11" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="G11" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="H11" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="I11" s="4" t="s">
+      <c r="C15" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="D15" s="11" t="s">
         <v>46</v>
       </c>
+      <c r="E15" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="F15" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="G15" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="H15" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="I15" s="11" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="E16" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="F16" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="G16" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="H16" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="I16" s="12" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="D17" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="E17" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="F17" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="G17" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="H17" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="I17" s="11" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="D18" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="E18" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="F18" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="G18" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="H18" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="I18" s="12" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C19" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="D19" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="E19" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="F19" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="G19" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="H19" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="I19" s="11" t="s">
+        <v>63</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:I2"/>
+  <mergeCells count="8">
+    <mergeCell ref="A2:B10"/>
+    <mergeCell ref="E2:E9"/>
+    <mergeCell ref="H3:H5"/>
+    <mergeCell ref="I3:I5"/>
+    <mergeCell ref="J3:J5"/>
+    <mergeCell ref="H6:H9"/>
+    <mergeCell ref="I6:I9"/>
+    <mergeCell ref="J6:J9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A2:J15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -1031,135 +1422,287 @@
     <col min="4" max="4" width="25" customWidth="1"/>
     <col min="5" max="6" width="16" customWidth="1"/>
     <col min="7" max="7" width="20" customWidth="1"/>
+    <col min="8" max="10" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="36" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-    </row>
-    <row r="2" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-    </row>
-    <row r="4" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>51</v>
+    <row r="2" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E2" s="4">
+        <v>3</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="G2" s="5">
+        <v>3</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="4"/>
+      <c r="F3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H3" s="7">
+        <v>3</v>
+      </c>
+      <c r="I3" s="7">
+        <v>0</v>
+      </c>
+      <c r="J3" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="5" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="6" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="7" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="D7" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="E7" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>61</v>
+      <c r="E4" s="4"/>
+      <c r="F4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H4" s="7"/>
+      <c r="I4" s="7"/>
+      <c r="J4" s="7"/>
+    </row>
+    <row r="5" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="4"/>
+      <c r="F5" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H5" s="7"/>
+      <c r="I5" s="7"/>
+      <c r="J5" s="7"/>
+    </row>
+    <row r="6" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" s="4"/>
+      <c r="H6" s="8">
+        <v>1</v>
+      </c>
+      <c r="I6" s="8">
+        <v>0</v>
+      </c>
+      <c r="J6" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="1"/>
+      <c r="B7" s="1"/>
+      <c r="C7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" s="4"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="8"/>
+      <c r="J7" s="8"/>
+    </row>
+    <row r="8" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="1"/>
+      <c r="B8" s="1"/>
+      <c r="C8" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" s="4"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+    </row>
+    <row r="9" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="1"/>
+      <c r="B9" s="1"/>
+      <c r="C9" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" s="4"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
+    </row>
+    <row r="10" ht="6" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="1"/>
+      <c r="B10" s="1"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="9"/>
+    </row>
+    <row r="11" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="12" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="D12" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="E12" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="F12" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="G12" s="10" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="F13" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="G13" s="11" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="D14" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="E14" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="F14" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="G14" s="12" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="D15" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="E15" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="F15" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="G15" s="11" t="s">
+        <v>79</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A2:G2"/>
+  <mergeCells count="8">
+    <mergeCell ref="A2:B10"/>
+    <mergeCell ref="E2:E9"/>
+    <mergeCell ref="H3:H5"/>
+    <mergeCell ref="I3:I5"/>
+    <mergeCell ref="J3:J5"/>
+    <mergeCell ref="H6:H9"/>
+    <mergeCell ref="I6:I9"/>
+    <mergeCell ref="J6:J9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A2:J19"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -1167,168 +1710,324 @@
     <col min="3" max="3" width="18" customWidth="1"/>
     <col min="4" max="4" width="55" customWidth="1"/>
     <col min="5" max="5" width="20" customWidth="1"/>
+    <col min="6" max="6" width="14" customWidth="1"/>
+    <col min="7" max="7" width="10" customWidth="1"/>
+    <col min="8" max="10" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="36" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-    </row>
-    <row r="2" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-    </row>
-    <row r="4" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="C4" s="3" t="s">
+    <row r="2" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="E2" s="4">
+        <v>7</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="G2" s="5">
+        <v>7</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="I2" s="6" t="s">
         <v>4</v>
       </c>
+      <c r="J2" s="6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="4"/>
+      <c r="F3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H3" s="7">
+        <v>7</v>
+      </c>
+      <c r="I3" s="7">
+        <v>0</v>
+      </c>
+      <c r="J3" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="2" t="s">
+        <v>9</v>
+      </c>
       <c r="D4" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="5" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="B5" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="E4" s="4"/>
+      <c r="F4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H4" s="7"/>
+      <c r="I4" s="7"/>
+      <c r="J4" s="7"/>
+    </row>
+    <row r="5" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="4"/>
+      <c r="F5" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H5" s="7"/>
+      <c r="I5" s="7"/>
+      <c r="J5" s="7"/>
+    </row>
+    <row r="6" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="6" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="B6" s="5" t="s">
+      <c r="D6" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" s="4"/>
+      <c r="H6" s="8">
+        <v>1</v>
+      </c>
+      <c r="I6" s="8">
+        <v>0</v>
+      </c>
+      <c r="J6" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="1"/>
+      <c r="B7" s="1"/>
+      <c r="C7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" s="4"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="8"/>
+      <c r="J7" s="8"/>
+    </row>
+    <row r="8" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="1"/>
+      <c r="B8" s="1"/>
+      <c r="C8" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" s="4"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+    </row>
+    <row r="9" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="1"/>
+      <c r="B9" s="1"/>
+      <c r="C9" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" s="4"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
+    </row>
+    <row r="10" ht="6" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="1"/>
+      <c r="B10" s="1"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+    </row>
+    <row r="11" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="12" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="C12" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="7" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="8" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="9" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="10" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="E10" s="5" t="s">
+      <c r="D12" s="10" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="11" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
+      <c r="E12" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D11" s="4" t="s">
+    </row>
+    <row r="13" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="B13" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="D13" s="11" t="s">
         <v>93</v>
       </c>
+      <c r="E13" s="11" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="D14" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="E14" s="12" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="D15" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="E15" s="11" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="E16" s="12" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="D17" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="E17" s="11" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="D18" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="E18" s="12" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C19" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="D19" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="E19" s="11" t="s">
+        <v>112</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A2:E2"/>
+  <mergeCells count="8">
+    <mergeCell ref="A2:B10"/>
+    <mergeCell ref="E2:E9"/>
+    <mergeCell ref="H3:H5"/>
+    <mergeCell ref="I3:I5"/>
+    <mergeCell ref="J3:J5"/>
+    <mergeCell ref="H6:H9"/>
+    <mergeCell ref="I6:I9"/>
+    <mergeCell ref="J6:J9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>